<commit_message>
Validate IFC object and TypeObject mappings separately
</commit_message>
<xml_diff>
--- a/templates/Strukturvorlage_DataDictionary_empty_public_v0.9.5.xlsx
+++ b/templates/Strukturvorlage_DataDictionary_empty_public_v0.9.5.xlsx
@@ -15226,7 +15226,7 @@
       </c>
       <c r="C105" s="193" t="inlineStr">
         <is>
-          <t>Der Objekttyp definiert die spezifischen Informationen zu einem Typ, die allen Instanzen dieses Typs gemeinsam sind.</t>
+          <t>Optionale IFC-TypeObject-Entität zur Dokumentation des Mapping-Umfangs. Leer = Mapping gilt nur für die Objektebene. Ausgefüllt = Mapping gilt zusätzlich für die angegebene Typebene; der Wert muss ein schema-konformes Paar mit „IfcObject Entity“ bilden (z. B. IfcTank → IfcTankType). Der PredefinedType wird separat erfasst und validiert.</t>
         </is>
       </c>
       <c r="F105" s="195" t="n"/>
@@ -18620,7 +18620,7 @@
       </c>
       <c r="Z2" s="60" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>optional</t>
         </is>
       </c>
       <c r="AA2" s="60" t="inlineStr">
@@ -19084,7 +19084,7 @@
       </c>
       <c r="Z6" s="104" t="inlineStr">
         <is>
-          <t>validated against IFC 4.3 entity identifiers</t>
+          <t>Leer = nur Objektebene; ausgefüllt = Mapping gilt auch für die angegebene Typebene; validiert gegen IFC 4.3 Objekt-/TypeObject-Paare</t>
         </is>
       </c>
       <c r="AA6" s="104" t="inlineStr">

</xml_diff>

<commit_message>
Support JSON lists for IFC set mappings
</commit_message>
<xml_diff>
--- a/templates/Strukturvorlage_DataDictionary_empty_public_v0.9.5.xlsx
+++ b/templates/Strukturvorlage_DataDictionary_empty_public_v0.9.5.xlsx
@@ -16248,7 +16248,7 @@
       </c>
       <c r="C140" s="193" t="inlineStr">
         <is>
-          <t>Beschreibt eine Liste von Merkmalen / Mebgeb für eine IFC-Entität. Merkmalssätze / Mengensätze, deren Struktur und Eigenschaften fest in der IFC-Spezifikation definiert sind.</t>
+          <t>Referenz auf einen IFC-Merkmals- oder Mengensatz. Ein Einzelwert wird direkt als Pset_*/Qto_*-Name oder zulässige absolute IRI erfasst. Mehrere Werte müssen als gültige JSON-Liste aus nicht leeren Strings mit doppelten Anführungszeichen erfasst werden, z. B. ["Pset_WallCommon", "Qto_WallBaseQuantities"]. Zeilenumbruch-, Semikolon- und einfache Kommalisten sind nicht zulässig.</t>
         </is>
       </c>
       <c r="F140" s="195" t="n"/>
@@ -20756,7 +20756,7 @@
       </c>
       <c r="X6" s="104" t="inlineStr">
         <is>
-          <t>validated against IFC 4.3 property/quantity set identifiers when IFC_URI is present</t>
+          <t>Ein Wert: Pset_* / Qto_* oder zulässige absolute IRI. Mehrere Werte: strikte JSON-Liste, z. B. ["Pset_WallCommon", "Qto_WallBaseQuantities"]; keine Zeilenumbruch-/Semikolonlisten.</t>
         </is>
       </c>
       <c r="Y6" s="104" t="inlineStr">

</xml_diff>